<commit_message>
Updating the Project CCR
</commit_message>
<xml_diff>
--- a/Document/1st_Year_Faculty_Credentials.xlsx
+++ b/Document/1st_Year_Faculty_Credentials.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -953,12 +953,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Mrs.A.VANI BERLIN</t>
+          <t>Mr.KUMARASAMY</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>mrsavaniberlin@ccr.edu</t>
+          <t>mrkumarasamy@ccr.edu</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Mr.KUMARASAMY</t>
+          <t>Mrs.VYSHNAVAI</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>mrkumarasamy@ccr.edu</t>
+          <t>mrsvyshnavai@ccr.edu</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -993,12 +993,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Mrs.VYSHNAVAI</t>
+          <t>Mr.ARAVIND</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>mrsvyshnavai@ccr.edu</t>
+          <t>mraravind@ccr.edu</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Mr.ARAVIND</t>
+          <t>Mr.VIJAYAKUMAR</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>mraravind@ccr.edu</t>
+          <t>mrvijayakumar@ccr.edu</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -1033,12 +1033,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Mr.VIJAYAKUMAR</t>
+          <t>Mr.KALAIMANII</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>mrvijayakumar@ccr.edu</t>
+          <t>mrkalaimanii@ccr.edu</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1053,12 +1053,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Mr.KALAIMANII</t>
+          <t>Mrs.AMUDHA</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>mrkalaimanii@ccr.edu</t>
+          <t>mrsamudha@ccr.edu</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -1073,12 +1073,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Mrs.AMUDHA</t>
+          <t>MS.GOPHIKA</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>mrsamudha@ccr.edu</t>
+          <t>msgophika@ccr.edu</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -1093,12 +1093,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>MS.GOPHIKA</t>
+          <t>Mr.KUMARASWAMY</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>msgophika@ccr.edu</t>
+          <t>mrkumaraswamy@ccr.edu</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -1113,12 +1113,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Mr.KUMARASWAMY</t>
+          <t>Mrs.R.SUMATHY</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>mrkumaraswamy@ccr.edu</t>
+          <t>mrsrsumathy@ccr.edu</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Mrs.R.SUMATHY</t>
+          <t>Mrs.G.REVATHY</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>mrsrsumathy@ccr.edu</t>
+          <t>mrsgrevathy@ccr.edu</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -1153,35 +1153,15 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Mrs.G.REVATHY</t>
+          <t>Mrs.ASHWINI</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>mrsgrevathy@ccr.edu</t>
+          <t>mrsashwini@ccr.edu</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>password123</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Mrs.ASHWINI</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>mrsashwini@ccr.edu</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>password123</t>
         </is>

</xml_diff>